<commit_message>
Add Cora as Blue Crew captain; new pairings with no-back-to-back constraint
- Cora (b13) added as 4th Blue Crew woman and captain
- Jay+Cora are the captain pair — 1 mixed game together in R7N
- All 3 regular couples (Alexis/Trevor, Carmela/Marv, Ivy/Pierre) play exactly 2 mixed each
- Women distribution: 1+2+2+2=7 ✓ (captain plays 1, others play 2)
- No-back-to-back constraint added: no player appears in two consecutive rounds
- Non-mixed men pool drops from 6 to 5; Rhon+Joe draw 4 games each
- Schedule.jsx: shows all 9 rounds dynamically with round times from config
- Scores.jsx: fixed to include round 9
- config.js: Hill Street Blues team name, Cora as captain, round times, updated RULES
- mockData.js: Cora b13 added, Alexis no longer captain, all 18 matches updated
- generate_template.py: Cora b13 added to example players
- ATHOPEN.md: Section 11 fully rewritten with new schedule, math, algorithm docs

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/BlueCrew_Pairings.xlsx
+++ b/docs/BlueCrew_Pairings.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,13 +69,18 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="007B4F00"/>
+      <color rgb="005E2CA5"/>
       <sz val="8"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007B4F00"/>
+      <sz val="8"/>
     </font>
     <font>
       <b val="1"/>
@@ -92,7 +97,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -117,6 +122,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF176"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EDE7F6"/>
       </patternFill>
     </fill>
     <fill>
@@ -171,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -209,15 +219,18 @@
     <xf numFmtId="0" fontId="8" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -232,19 +245,31 @@
     <xf numFmtId="0" fontId="9" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -265,13 +290,22 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -639,7 +673,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -650,6 +684,7 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -692,6 +727,11 @@
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="3" t="inlineStr"/>
@@ -718,6 +758,7 @@
           <t>Player 2</t>
         </is>
       </c>
+      <c r="I3" s="3" t="inlineStr"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="4" t="n">
@@ -725,7 +766,7 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>8:30 am</t>
+          <t>8:30 AM</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
@@ -750,14 +791,15 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Arman</t>
+          <t>Joe</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Rhon</t>
-        </is>
-      </c>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="4" t="n">
@@ -765,7 +807,7 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>8:30 am</t>
+          <t>8:30 AM</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -790,14 +832,15 @@
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Richard</t>
+          <t>Rhon</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Jon</t>
-        </is>
-      </c>
+          <t>Trevor</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="4" t="n">
@@ -805,7 +848,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>8:50 am</t>
+          <t>8:50 AM</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -830,14 +873,15 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Joe</t>
+          <t>Arman</t>
         </is>
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Arman</t>
-        </is>
-      </c>
+          <t>Pierre</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="4" t="n">
@@ -845,7 +889,7 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>8:50 am</t>
+          <t>8:50 AM</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -870,14 +914,15 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Jay</t>
+          <t>Jon</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
         <is>
-          <t>Rhon</t>
-        </is>
-      </c>
+          <t>Marv</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="4" t="n">
@@ -885,7 +930,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>9:15 am</t>
+          <t>9:15 AM</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -910,14 +955,15 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Richard</t>
+          <t>Joe</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Jay</t>
-        </is>
-      </c>
+          <t>Rhon</t>
+        </is>
+      </c>
+      <c r="I8" s="5" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="4" t="n">
@@ -925,7 +971,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>9:15 am</t>
+          <t>9:15 AM</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
@@ -950,14 +996,15 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Arman</t>
+          <t>Richard</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Pierre</t>
-        </is>
-      </c>
+          <t>Jay</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="6" t="n">
@@ -965,7 +1012,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>9:40 am</t>
+          <t>9:40 AM</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -990,14 +1037,15 @@
       </c>
       <c r="G10" s="7" t="inlineStr">
         <is>
-          <t>Marv</t>
+          <t>Pierre</t>
         </is>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>Carmela</t>
-        </is>
-      </c>
+          <t>Ivy</t>
+        </is>
+      </c>
+      <c r="I10" s="7" t="inlineStr"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -1005,7 +1053,7 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>9:40 am</t>
+          <t>9:40 AM</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
@@ -1030,14 +1078,15 @@
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Trevor</t>
+          <t>Marv</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>Alexis</t>
-        </is>
-      </c>
+          <t>Carmela</t>
+        </is>
+      </c>
+      <c r="I11" s="7" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="6" t="n">
@@ -1045,7 +1094,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>10:10 am</t>
+          <t>10:10 AM</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -1070,14 +1119,15 @@
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Marv</t>
+          <t>Trevor</t>
         </is>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>Carmela</t>
-        </is>
-      </c>
+          <t>Alexis</t>
+        </is>
+      </c>
+      <c r="I12" s="7" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="4" t="n">
@@ -1085,7 +1135,7 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>10:10 am</t>
+          <t>10:10 AM</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
@@ -1110,14 +1160,15 @@
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Richard</t>
+          <t>Jay</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
         <is>
-          <t>Arman</t>
-        </is>
-      </c>
+          <t>Rhon</t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="4" t="n">
@@ -1125,7 +1176,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>10:30 am</t>
+          <t>10:30 AM</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1150,14 +1201,15 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Jay</t>
+          <t>Richard</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>Joe</t>
-        </is>
-      </c>
+          <t>Arman</t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="4" t="n">
@@ -1165,7 +1217,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>10:30 am</t>
+          <t>10:30 AM</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
@@ -1190,14 +1242,15 @@
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
+          <t>Joe</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
           <t>Jon</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
-        <is>
-          <t>Trevor</t>
-        </is>
-      </c>
+      <c r="I15" s="5" t="inlineStr"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="6" t="n">
@@ -1205,7 +1258,7 @@
       </c>
       <c r="B16" s="6" t="inlineStr">
         <is>
-          <t>11:00 am</t>
+          <t>11:00 AM</t>
         </is>
       </c>
       <c r="C16" s="6" t="inlineStr">
@@ -1230,14 +1283,15 @@
       </c>
       <c r="G16" s="7" t="inlineStr">
         <is>
-          <t>Trevor</t>
+          <t>Pierre</t>
         </is>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>Alexis</t>
-        </is>
-      </c>
+          <t>Ivy</t>
+        </is>
+      </c>
+      <c r="I16" s="7" t="inlineStr"/>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -1245,7 +1299,7 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>11:00 am</t>
+          <t>11:00 AM</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
@@ -1270,12 +1324,17 @@
       </c>
       <c r="G17" s="7" t="inlineStr">
         <is>
-          <t>Pierre</t>
+          <t>Jay</t>
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>Ivy</t>
+          <t>Cora</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>Captain's game ★</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1344,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>11:30 am</t>
+          <t>11:30 AM</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -1310,14 +1369,15 @@
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Richard</t>
+          <t>Arman</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Rhon</t>
-        </is>
-      </c>
+          <t>Joe</t>
+        </is>
+      </c>
+      <c r="I18" s="5" t="inlineStr"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="4" t="n">
@@ -1325,7 +1385,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>11:30 am</t>
+          <t>11:30 AM</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -1350,7 +1410,7 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Joe</t>
+          <t>Rhon</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -1358,6 +1418,7 @@
           <t>Jon</t>
         </is>
       </c>
+      <c r="I19" s="5" t="inlineStr"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="6" t="n">
@@ -1390,14 +1451,15 @@
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>Pierre</t>
+          <t>Trevor</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>Ivy</t>
-        </is>
-      </c>
+          <t>Alexis</t>
+        </is>
+      </c>
+      <c r="I20" s="7" t="inlineStr"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="6" t="n">
@@ -1438,10 +1500,11 @@
           <t>Carmela</t>
         </is>
       </c>
+      <c r="I21" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A1:I1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1453,11 +1516,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q16"/>
+  <dimension ref="A1:R17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="7" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
@@ -1470,19 +1533,20 @@
     <col width="7" customWidth="1" min="12" max="12"/>
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="8" t="inlineStr">
         <is>
-          <t>Blue Crew (JPL Team) — Pairings Matrix   (X = Men's Doubles  |  M★ = Mixed Doubles)</t>
+          <t>Blue Crew (JPL Team) — Pairings Matrix   (X = Men's Doubles  |  M★ = Mixed Doubles  |  C★ = Captain's game)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Couples: Trevor ↔ Alexis  ·  Marv ↔ Carmela  ·  Pierre ↔ Ivy    |    Pairings randomised (no skill ranking)</t>
+          <t>Captain: Cora (1 game w/ Jay)  ·  Couples: Trevor↔Alexis, Marv↔Carmela, Pierre↔Ivy  |  No back-to-back games</t>
         </is>
       </c>
     </row>
@@ -1500,579 +1564,634 @@
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
+          <t>Cora
+(C★)</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
           <t>Alexis
-(F★)</t>
-        </is>
-      </c>
-      <c r="D4" s="11" t="inlineStr">
+(F)</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
         <is>
           <t>Carmela
-(F★)</t>
-        </is>
-      </c>
-      <c r="E4" s="11" t="inlineStr">
+(F)</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
         <is>
           <t>Ivy
-(F★)</t>
-        </is>
-      </c>
-      <c r="F4" s="12" t="inlineStr">
+(F)</t>
+        </is>
+      </c>
+      <c r="G4" s="13" t="inlineStr">
         <is>
           <t>Jay
 (M)</t>
         </is>
       </c>
-      <c r="G4" s="12" t="inlineStr">
+      <c r="H4" s="13" t="inlineStr">
         <is>
           <t>Marv
 (M)</t>
         </is>
       </c>
-      <c r="H4" s="12" t="inlineStr">
+      <c r="I4" s="13" t="inlineStr">
         <is>
           <t>Arman
 (M)</t>
         </is>
       </c>
-      <c r="I4" s="12" t="inlineStr">
+      <c r="J4" s="13" t="inlineStr">
         <is>
           <t>Jon
 (M)</t>
         </is>
       </c>
-      <c r="J4" s="12" t="inlineStr">
+      <c r="K4" s="13" t="inlineStr">
         <is>
           <t>Trevor
 (M)</t>
         </is>
       </c>
-      <c r="K4" s="12" t="inlineStr">
+      <c r="L4" s="13" t="inlineStr">
         <is>
           <t>Richard
 (M)</t>
         </is>
       </c>
-      <c r="L4" s="12" t="inlineStr">
+      <c r="M4" s="13" t="inlineStr">
         <is>
           <t>Rhon
 (M)</t>
         </is>
       </c>
-      <c r="M4" s="12" t="inlineStr">
+      <c r="N4" s="13" t="inlineStr">
         <is>
           <t>Joe
 (M)</t>
         </is>
       </c>
-      <c r="N4" s="12" t="inlineStr">
+      <c r="O4" s="13" t="inlineStr">
         <is>
           <t>Pierre
 (M)</t>
         </is>
       </c>
-      <c r="O4" s="10" t="inlineStr">
+      <c r="P4" s="10" t="inlineStr">
         <is>
           <t>Games</t>
         </is>
       </c>
-      <c r="P4" s="10" t="inlineStr">
+      <c r="Q4" s="10" t="inlineStr">
         <is>
           <t>Mix★</t>
         </is>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="13" t="n">
+      <c r="A5" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>Alexis (F)</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="n"/>
-      <c r="D5" s="16" t="n"/>
-      <c r="E5" s="16" t="n"/>
-      <c r="F5" s="16" t="n"/>
-      <c r="G5" s="16" t="n"/>
-      <c r="H5" s="16" t="n"/>
-      <c r="I5" s="16" t="n"/>
-      <c r="J5" s="17" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Cora (Captain)</t>
+        </is>
+      </c>
+      <c r="C5" s="16" t="n"/>
+      <c r="D5" s="17" t="n"/>
+      <c r="E5" s="17" t="n"/>
+      <c r="F5" s="17" t="n"/>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>C★
+R7-N</t>
+        </is>
+      </c>
+      <c r="H5" s="17" t="n"/>
+      <c r="I5" s="17" t="n"/>
+      <c r="J5" s="17" t="n"/>
+      <c r="K5" s="17" t="n"/>
+      <c r="L5" s="17" t="n"/>
+      <c r="M5" s="17" t="n"/>
+      <c r="N5" s="17" t="n"/>
+      <c r="O5" s="17" t="n"/>
+      <c r="P5" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="21" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>Alexis</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="n"/>
+      <c r="D6" s="16" t="n"/>
+      <c r="E6" s="17" t="n"/>
+      <c r="F6" s="17" t="n"/>
+      <c r="G6" s="17" t="n"/>
+      <c r="H6" s="17" t="n"/>
+      <c r="I6" s="17" t="n"/>
+      <c r="J6" s="17" t="n"/>
+      <c r="K6" s="23" t="inlineStr">
+        <is>
+          <t>M★
+R9-S</t>
+        </is>
+      </c>
+      <c r="L6" s="17" t="n"/>
+      <c r="M6" s="17" t="n"/>
+      <c r="N6" s="17" t="n"/>
+      <c r="O6" s="17" t="n"/>
+      <c r="P6" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q6" s="20" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="21" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>Carmela</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="n"/>
+      <c r="D7" s="17" t="n"/>
+      <c r="E7" s="16" t="n"/>
+      <c r="F7" s="17" t="n"/>
+      <c r="G7" s="17" t="n"/>
+      <c r="H7" s="23" t="inlineStr">
+        <is>
+          <t>M★
+R9-N</t>
+        </is>
+      </c>
+      <c r="I7" s="17" t="n"/>
+      <c r="J7" s="17" t="n"/>
+      <c r="K7" s="17" t="n"/>
+      <c r="L7" s="17" t="n"/>
+      <c r="M7" s="17" t="n"/>
+      <c r="N7" s="17" t="n"/>
+      <c r="O7" s="17" t="n"/>
+      <c r="P7" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q7" s="20" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="21" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>Ivy</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="n"/>
+      <c r="D8" s="17" t="n"/>
+      <c r="E8" s="17" t="n"/>
+      <c r="F8" s="16" t="n"/>
+      <c r="G8" s="17" t="n"/>
+      <c r="H8" s="17" t="n"/>
+      <c r="I8" s="17" t="n"/>
+      <c r="J8" s="17" t="n"/>
+      <c r="K8" s="17" t="n"/>
+      <c r="L8" s="17" t="n"/>
+      <c r="M8" s="17" t="n"/>
+      <c r="N8" s="17" t="n"/>
+      <c r="O8" s="23" t="inlineStr">
         <is>
           <t>M★
 R7-S</t>
         </is>
       </c>
-      <c r="K5" s="16" t="n"/>
-      <c r="L5" s="16" t="n"/>
-      <c r="M5" s="16" t="n"/>
-      <c r="N5" s="16" t="n"/>
-      <c r="O5" s="18" t="n">
+      <c r="P8" s="24" t="n">
         <v>2</v>
       </c>
-      <c r="P5" s="19" t="n">
+      <c r="Q8" s="20" t="n">
         <v>2</v>
       </c>
     </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>Carmela (F)</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="n"/>
-      <c r="D6" s="15" t="n"/>
-      <c r="E6" s="16" t="n"/>
-      <c r="F6" s="16" t="n"/>
-      <c r="G6" s="17" t="inlineStr">
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Jay</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>C★
+R7-N</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="n"/>
+      <c r="E9" s="17" t="n"/>
+      <c r="F9" s="17" t="n"/>
+      <c r="G9" s="16" t="n"/>
+      <c r="H9" s="17" t="n"/>
+      <c r="I9" s="17" t="n"/>
+      <c r="J9" s="17" t="n"/>
+      <c r="K9" s="17" t="n"/>
+      <c r="L9" s="27" t="inlineStr">
+        <is>
+          <t>X
+R3-N</t>
+        </is>
+      </c>
+      <c r="M9" s="27" t="inlineStr">
+        <is>
+          <t>X
+R5-N</t>
+        </is>
+      </c>
+      <c r="N9" s="17" t="n"/>
+      <c r="O9" s="17" t="n"/>
+      <c r="P9" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q9" s="20" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="25" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Marv</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="n"/>
+      <c r="D10" s="17" t="n"/>
+      <c r="E10" s="23" t="inlineStr">
         <is>
           <t>M★
 R9-N</t>
         </is>
       </c>
-      <c r="H6" s="16" t="n"/>
-      <c r="I6" s="16" t="n"/>
-      <c r="J6" s="16" t="n"/>
-      <c r="K6" s="16" t="n"/>
-      <c r="L6" s="16" t="n"/>
-      <c r="M6" s="16" t="n"/>
-      <c r="N6" s="16" t="n"/>
-      <c r="O6" s="18" t="n">
+      <c r="F10" s="17" t="n"/>
+      <c r="G10" s="17" t="n"/>
+      <c r="H10" s="16" t="n"/>
+      <c r="I10" s="17" t="n"/>
+      <c r="J10" s="27" t="inlineStr">
+        <is>
+          <t>X
+R2-N</t>
+        </is>
+      </c>
+      <c r="K10" s="17" t="n"/>
+      <c r="L10" s="17" t="n"/>
+      <c r="M10" s="17" t="n"/>
+      <c r="N10" s="17" t="n"/>
+      <c r="O10" s="17" t="n"/>
+      <c r="P10" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="P6" s="19" t="n">
+      <c r="Q10" s="20" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="25" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="26" t="inlineStr">
+        <is>
+          <t>Arman</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="n"/>
+      <c r="D11" s="17" t="n"/>
+      <c r="E11" s="17" t="n"/>
+      <c r="F11" s="17" t="n"/>
+      <c r="G11" s="17" t="n"/>
+      <c r="H11" s="17" t="n"/>
+      <c r="I11" s="16" t="n"/>
+      <c r="J11" s="17" t="n"/>
+      <c r="K11" s="17" t="n"/>
+      <c r="L11" s="27" t="inlineStr">
+        <is>
+          <t>X
+R6-S</t>
+        </is>
+      </c>
+      <c r="M11" s="17" t="n"/>
+      <c r="N11" s="27" t="inlineStr">
+        <is>
+          <t>X
+R8-S</t>
+        </is>
+      </c>
+      <c r="O11" s="27" t="inlineStr">
+        <is>
+          <t>X
+R2-S</t>
+        </is>
+      </c>
+      <c r="P11" s="28" t="n">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="13" t="n">
+      <c r="Q11" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Jon</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="n"/>
+      <c r="D12" s="17" t="n"/>
+      <c r="E12" s="17" t="n"/>
+      <c r="F12" s="17" t="n"/>
+      <c r="G12" s="17" t="n"/>
+      <c r="H12" s="27" t="inlineStr">
+        <is>
+          <t>X
+R2-N</t>
+        </is>
+      </c>
+      <c r="I12" s="17" t="n"/>
+      <c r="J12" s="16" t="n"/>
+      <c r="K12" s="17" t="n"/>
+      <c r="L12" s="17" t="n"/>
+      <c r="M12" s="27" t="inlineStr">
+        <is>
+          <t>X
+R8-N</t>
+        </is>
+      </c>
+      <c r="N12" s="27" t="inlineStr">
+        <is>
+          <t>X
+R6-N</t>
+        </is>
+      </c>
+      <c r="O12" s="17" t="n"/>
+      <c r="P12" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>Ivy (F)</t>
-        </is>
-      </c>
-      <c r="C7" s="16" t="n"/>
-      <c r="D7" s="16" t="n"/>
-      <c r="E7" s="15" t="n"/>
-      <c r="F7" s="16" t="n"/>
-      <c r="G7" s="16" t="n"/>
-      <c r="H7" s="16" t="n"/>
-      <c r="I7" s="16" t="n"/>
-      <c r="J7" s="16" t="n"/>
-      <c r="K7" s="16" t="n"/>
-      <c r="L7" s="16" t="n"/>
-      <c r="M7" s="16" t="n"/>
-      <c r="N7" s="17" t="inlineStr">
+      <c r="Q12" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="25" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>Trevor</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="n"/>
+      <c r="D13" s="23" t="inlineStr">
         <is>
           <t>M★
 R9-S</t>
         </is>
       </c>
-      <c r="O7" s="18" t="n">
+      <c r="E13" s="17" t="n"/>
+      <c r="F13" s="17" t="n"/>
+      <c r="G13" s="17" t="n"/>
+      <c r="H13" s="17" t="n"/>
+      <c r="I13" s="17" t="n"/>
+      <c r="J13" s="17" t="n"/>
+      <c r="K13" s="16" t="n"/>
+      <c r="L13" s="17" t="n"/>
+      <c r="M13" s="27" t="inlineStr">
+        <is>
+          <t>X
+R1-N</t>
+        </is>
+      </c>
+      <c r="N13" s="17" t="n"/>
+      <c r="O13" s="17" t="n"/>
+      <c r="P13" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q13" s="20" t="n">
         <v>2</v>
       </c>
-      <c r="P7" s="19" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="20" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="21" t="inlineStr">
-        <is>
-          <t>Jay (M)</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="n"/>
-      <c r="D8" s="16" t="n"/>
-      <c r="E8" s="16" t="n"/>
-      <c r="F8" s="15" t="n"/>
-      <c r="G8" s="16" t="n"/>
-      <c r="H8" s="16" t="n"/>
-      <c r="I8" s="16" t="n"/>
-      <c r="J8" s="16" t="n"/>
-      <c r="K8" s="22" t="inlineStr">
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="n"/>
+      <c r="D14" s="17" t="n"/>
+      <c r="E14" s="17" t="n"/>
+      <c r="F14" s="17" t="n"/>
+      <c r="G14" s="27" t="inlineStr">
+        <is>
+          <t>X
+R3-N</t>
+        </is>
+      </c>
+      <c r="H14" s="17" t="n"/>
+      <c r="I14" s="27" t="inlineStr">
+        <is>
+          <t>X
+R6-S</t>
+        </is>
+      </c>
+      <c r="J14" s="17" t="n"/>
+      <c r="K14" s="17" t="n"/>
+      <c r="L14" s="16" t="n"/>
+      <c r="M14" s="17" t="n"/>
+      <c r="N14" s="27" t="inlineStr">
+        <is>
+          <t>X
+R1-S</t>
+        </is>
+      </c>
+      <c r="O14" s="17" t="n"/>
+      <c r="P14" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q14" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="25" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>Rhon</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="n"/>
+      <c r="D15" s="17" t="n"/>
+      <c r="E15" s="17" t="n"/>
+      <c r="F15" s="17" t="n"/>
+      <c r="G15" s="27" t="inlineStr">
+        <is>
+          <t>X
+R5-N</t>
+        </is>
+      </c>
+      <c r="H15" s="17" t="n"/>
+      <c r="I15" s="17" t="n"/>
+      <c r="J15" s="27" t="inlineStr">
+        <is>
+          <t>X
+R8-N</t>
+        </is>
+      </c>
+      <c r="K15" s="27" t="inlineStr">
+        <is>
+          <t>X
+R1-N</t>
+        </is>
+      </c>
+      <c r="L15" s="17" t="n"/>
+      <c r="M15" s="16" t="n"/>
+      <c r="N15" s="27" t="inlineStr">
         <is>
           <t>X
 R3-S</t>
         </is>
       </c>
-      <c r="L8" s="22" t="inlineStr">
+      <c r="O15" s="17" t="n"/>
+      <c r="P15" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q15" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>Joe</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="n"/>
+      <c r="D16" s="17" t="n"/>
+      <c r="E16" s="17" t="n"/>
+      <c r="F16" s="17" t="n"/>
+      <c r="G16" s="17" t="n"/>
+      <c r="H16" s="17" t="n"/>
+      <c r="I16" s="27" t="inlineStr">
         <is>
           <t>X
-R2-N</t>
-        </is>
-      </c>
-      <c r="M8" s="22" t="inlineStr">
+R8-S</t>
+        </is>
+      </c>
+      <c r="J16" s="27" t="inlineStr">
         <is>
           <t>X
-R6-S</t>
-        </is>
-      </c>
-      <c r="N8" s="16" t="n"/>
-      <c r="O8" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="P8" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="21" t="inlineStr">
-        <is>
-          <t>Marv (M)</t>
-        </is>
-      </c>
-      <c r="C9" s="16" t="n"/>
-      <c r="D9" s="17" t="inlineStr">
-        <is>
-          <t>M★
-R9-N</t>
-        </is>
-      </c>
-      <c r="E9" s="16" t="n"/>
-      <c r="F9" s="16" t="n"/>
-      <c r="G9" s="15" t="n"/>
-      <c r="H9" s="16" t="n"/>
-      <c r="I9" s="16" t="n"/>
-      <c r="J9" s="16" t="n"/>
-      <c r="K9" s="16" t="n"/>
-      <c r="L9" s="16" t="n"/>
-      <c r="M9" s="16" t="n"/>
-      <c r="N9" s="16" t="n"/>
-      <c r="O9" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="P9" s="19" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="21" t="inlineStr">
-        <is>
-          <t>Arman (M)</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="n"/>
-      <c r="D10" s="16" t="n"/>
-      <c r="E10" s="16" t="n"/>
-      <c r="F10" s="16" t="n"/>
-      <c r="G10" s="16" t="n"/>
-      <c r="H10" s="15" t="n"/>
-      <c r="I10" s="16" t="n"/>
-      <c r="J10" s="16" t="n"/>
-      <c r="K10" s="22" t="inlineStr">
-        <is>
-          <t>X
-R5-N</t>
-        </is>
-      </c>
-      <c r="L10" s="22" t="inlineStr">
+R6-N</t>
+        </is>
+      </c>
+      <c r="K16" s="17" t="n"/>
+      <c r="L16" s="27" t="inlineStr">
         <is>
           <t>X
 R1-S</t>
         </is>
       </c>
-      <c r="M10" s="22" t="inlineStr">
+      <c r="M16" s="27" t="inlineStr">
+        <is>
+          <t>X
+R3-S</t>
+        </is>
+      </c>
+      <c r="N16" s="16" t="n"/>
+      <c r="O16" s="17" t="n"/>
+      <c r="P16" s="30" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q16" s="29" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="25" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="26" t="inlineStr">
+        <is>
+          <t>Pierre</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="n"/>
+      <c r="D17" s="17" t="n"/>
+      <c r="E17" s="17" t="n"/>
+      <c r="F17" s="23" t="inlineStr">
+        <is>
+          <t>M★
+R7-S</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="n"/>
+      <c r="H17" s="17" t="n"/>
+      <c r="I17" s="27" t="inlineStr">
         <is>
           <t>X
 R2-S</t>
         </is>
       </c>
-      <c r="N10" s="22" t="inlineStr">
-        <is>
-          <t>X
-R3-N</t>
-        </is>
-      </c>
-      <c r="O10" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="P10" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="20" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="21" t="inlineStr">
-        <is>
-          <t>Jon (M)</t>
-        </is>
-      </c>
-      <c r="C11" s="16" t="n"/>
-      <c r="D11" s="16" t="n"/>
-      <c r="E11" s="16" t="n"/>
-      <c r="F11" s="16" t="n"/>
-      <c r="G11" s="16" t="n"/>
-      <c r="H11" s="16" t="n"/>
-      <c r="I11" s="15" t="n"/>
-      <c r="J11" s="22" t="inlineStr">
-        <is>
-          <t>X
-R6-N</t>
-        </is>
-      </c>
-      <c r="K11" s="22" t="inlineStr">
-        <is>
-          <t>X
-R1-N</t>
-        </is>
-      </c>
-      <c r="L11" s="16" t="n"/>
-      <c r="M11" s="22" t="inlineStr">
-        <is>
-          <t>X
-R8-N</t>
-        </is>
-      </c>
-      <c r="N11" s="16" t="n"/>
-      <c r="O11" s="23" t="n">
+      <c r="J17" s="17" t="n"/>
+      <c r="K17" s="17" t="n"/>
+      <c r="L17" s="17" t="n"/>
+      <c r="M17" s="17" t="n"/>
+      <c r="N17" s="17" t="n"/>
+      <c r="O17" s="16" t="n"/>
+      <c r="P17" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="P11" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="20" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="21" t="inlineStr">
-        <is>
-          <t>Trevor (M)</t>
-        </is>
-      </c>
-      <c r="C12" s="17" t="inlineStr">
-        <is>
-          <t>M★
-R7-S</t>
-        </is>
-      </c>
-      <c r="D12" s="16" t="n"/>
-      <c r="E12" s="16" t="n"/>
-      <c r="F12" s="16" t="n"/>
-      <c r="G12" s="16" t="n"/>
-      <c r="H12" s="16" t="n"/>
-      <c r="I12" s="22" t="inlineStr">
-        <is>
-          <t>X
-R6-N</t>
-        </is>
-      </c>
-      <c r="J12" s="15" t="n"/>
-      <c r="K12" s="16" t="n"/>
-      <c r="L12" s="16" t="n"/>
-      <c r="M12" s="16" t="n"/>
-      <c r="N12" s="16" t="n"/>
-      <c r="O12" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="P12" s="19" t="n">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="20" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="21" t="inlineStr">
-        <is>
-          <t>Richard (M)</t>
-        </is>
-      </c>
-      <c r="C13" s="16" t="n"/>
-      <c r="D13" s="16" t="n"/>
-      <c r="E13" s="16" t="n"/>
-      <c r="F13" s="22" t="inlineStr">
-        <is>
-          <t>X
-R3-S</t>
-        </is>
-      </c>
-      <c r="G13" s="16" t="n"/>
-      <c r="H13" s="22" t="inlineStr">
-        <is>
-          <t>X
-R5-N</t>
-        </is>
-      </c>
-      <c r="I13" s="22" t="inlineStr">
-        <is>
-          <t>X
-R1-N</t>
-        </is>
-      </c>
-      <c r="J13" s="16" t="n"/>
-      <c r="K13" s="15" t="n"/>
-      <c r="L13" s="22" t="inlineStr">
-        <is>
-          <t>X
-R8-S</t>
-        </is>
-      </c>
-      <c r="M13" s="16" t="n"/>
-      <c r="N13" s="16" t="n"/>
-      <c r="O13" s="25" t="n">
-        <v>4</v>
-      </c>
-      <c r="P13" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="20" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="21" t="inlineStr">
-        <is>
-          <t>Rhon (M)</t>
-        </is>
-      </c>
-      <c r="C14" s="16" t="n"/>
-      <c r="D14" s="16" t="n"/>
-      <c r="E14" s="16" t="n"/>
-      <c r="F14" s="22" t="inlineStr">
-        <is>
-          <t>X
-R2-N</t>
-        </is>
-      </c>
-      <c r="G14" s="16" t="n"/>
-      <c r="H14" s="22" t="inlineStr">
-        <is>
-          <t>X
-R1-S</t>
-        </is>
-      </c>
-      <c r="I14" s="16" t="n"/>
-      <c r="J14" s="16" t="n"/>
-      <c r="K14" s="22" t="inlineStr">
-        <is>
-          <t>X
-R8-S</t>
-        </is>
-      </c>
-      <c r="L14" s="15" t="n"/>
-      <c r="M14" s="16" t="n"/>
-      <c r="N14" s="16" t="n"/>
-      <c r="O14" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="P14" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="20" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="21" t="inlineStr">
-        <is>
-          <t>Joe (M)</t>
-        </is>
-      </c>
-      <c r="C15" s="16" t="n"/>
-      <c r="D15" s="16" t="n"/>
-      <c r="E15" s="16" t="n"/>
-      <c r="F15" s="22" t="inlineStr">
-        <is>
-          <t>X
-R6-S</t>
-        </is>
-      </c>
-      <c r="G15" s="16" t="n"/>
-      <c r="H15" s="22" t="inlineStr">
-        <is>
-          <t>X
-R2-S</t>
-        </is>
-      </c>
-      <c r="I15" s="22" t="inlineStr">
-        <is>
-          <t>X
-R8-N</t>
-        </is>
-      </c>
-      <c r="J15" s="16" t="n"/>
-      <c r="K15" s="16" t="n"/>
-      <c r="L15" s="16" t="n"/>
-      <c r="M15" s="15" t="n"/>
-      <c r="N15" s="16" t="n"/>
-      <c r="O15" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="P15" s="24" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="20" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="21" t="inlineStr">
-        <is>
-          <t>Pierre (M)</t>
-        </is>
-      </c>
-      <c r="C16" s="16" t="n"/>
-      <c r="D16" s="16" t="n"/>
-      <c r="E16" s="17" t="inlineStr">
-        <is>
-          <t>M★
-R9-S</t>
-        </is>
-      </c>
-      <c r="F16" s="16" t="n"/>
-      <c r="G16" s="16" t="n"/>
-      <c r="H16" s="22" t="inlineStr">
-        <is>
-          <t>X
-R3-N</t>
-        </is>
-      </c>
-      <c r="I16" s="16" t="n"/>
-      <c r="J16" s="16" t="n"/>
-      <c r="K16" s="16" t="n"/>
-      <c r="L16" s="16" t="n"/>
-      <c r="M16" s="16" t="n"/>
-      <c r="N16" s="15" t="n"/>
-      <c r="O16" s="23" t="n">
-        <v>3</v>
-      </c>
-      <c r="P16" s="19" t="n">
+      <c r="Q17" s="20" t="n">
         <v>2</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:Q2"/>
-    <mergeCell ref="A1:Q1"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2084,466 +2203,500 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="72" customWidth="1" min="8" max="8"/>
+    <col width="80" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="26" t="inlineStr">
-        <is>
-          <t>Rank</t>
-        </is>
-      </c>
-      <c r="B1" s="26" t="inlineStr">
+      <c r="A1" s="31" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="31" t="inlineStr">
         <is>
           <t>Player</t>
         </is>
       </c>
-      <c r="C1" s="26" t="inlineStr">
+      <c r="C1" s="31" t="inlineStr">
         <is>
           <t>Gender</t>
         </is>
       </c>
-      <c r="D1" s="26" t="inlineStr">
-        <is>
-          <t>Couple Partner</t>
-        </is>
-      </c>
-      <c r="E1" s="26" t="inlineStr">
+      <c r="D1" s="31" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="E1" s="31" t="inlineStr">
         <is>
           <t>Total Games</t>
         </is>
       </c>
-      <c r="F1" s="26" t="inlineStr">
-        <is>
-          <t>Men's Doubles</t>
-        </is>
-      </c>
-      <c r="G1" s="26" t="inlineStr">
+      <c r="F1" s="31" t="inlineStr">
+        <is>
+          <t>Men's Dbl</t>
+        </is>
+      </c>
+      <c r="G1" s="31" t="inlineStr">
         <is>
           <t>Mixed★</t>
         </is>
       </c>
-      <c r="H1" s="26" t="inlineStr">
-        <is>
-          <t>All Partners (round)</t>
+      <c r="H1" s="31" t="inlineStr">
+        <is>
+          <t>Games in order (round)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="27" t="n">
+      <c r="A2" s="32" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="28" t="inlineStr">
+      <c r="B2" s="33" t="inlineStr">
+        <is>
+          <t>Cora</t>
+        </is>
+      </c>
+      <c r="C2" s="32" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D2" s="32" t="inlineStr">
+        <is>
+          <t>Captain</t>
+        </is>
+      </c>
+      <c r="E2" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="34" t="inlineStr">
+        <is>
+          <t>R7★ w/Jay</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="36" t="inlineStr">
         <is>
           <t>Alexis</t>
         </is>
       </c>
-      <c r="C2" s="27" t="inlineStr">
+      <c r="C3" s="35" t="inlineStr">
         <is>
           <t>F</t>
         </is>
       </c>
-      <c r="D2" s="27" t="inlineStr">
+      <c r="D3" s="35" t="inlineStr">
+        <is>
+          <t>Couple</t>
+        </is>
+      </c>
+      <c r="E3" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" s="37" t="inlineStr">
+        <is>
+          <t>R5★ w/Trevor,  R9★ w/Trevor</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="35" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="36" t="inlineStr">
+        <is>
+          <t>Carmela</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>Couple</t>
+        </is>
+      </c>
+      <c r="E4" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" s="37" t="inlineStr">
+        <is>
+          <t>R4★ w/Marv,  R9★ w/Marv</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="36" t="inlineStr">
+        <is>
+          <t>Ivy</t>
+        </is>
+      </c>
+      <c r="C5" s="35" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="D5" s="35" t="inlineStr">
+        <is>
+          <t>Couple</t>
+        </is>
+      </c>
+      <c r="E5" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="35" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" s="37" t="inlineStr">
+        <is>
+          <t>R4★ w/Pierre,  R7★ w/Pierre</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="39" t="inlineStr">
+        <is>
+          <t>Jay</t>
+        </is>
+      </c>
+      <c r="C6" s="38" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D6" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="F6" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="G6" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" s="40" t="inlineStr">
+        <is>
+          <t>R3 w/Richard,  R5 w/Rhon,  R7★ w/Cora</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="38" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="39" t="inlineStr">
+        <is>
+          <t>Marv</t>
+        </is>
+      </c>
+      <c r="C7" s="38" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D7" s="38" t="inlineStr">
+        <is>
+          <t>Couple</t>
+        </is>
+      </c>
+      <c r="E7" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="40" t="inlineStr">
+        <is>
+          <t>R2 w/Jon,  R4★ w/Carmela,  R9★ w/Carmela</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="38" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="39" t="inlineStr">
+        <is>
+          <t>Arman</t>
+        </is>
+      </c>
+      <c r="C8" s="38" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D8" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="40" t="inlineStr">
+        <is>
+          <t>R2 w/Pierre,  R6 w/Richard,  R8 w/Joe</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="38" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="39" t="inlineStr">
+        <is>
+          <t>Jon</t>
+        </is>
+      </c>
+      <c r="C9" s="38" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D9" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="40" t="inlineStr">
+        <is>
+          <t>R2 w/Marv,  R6 w/Joe,  R8 w/Rhon</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="38" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="39" t="inlineStr">
         <is>
           <t>Trevor</t>
         </is>
       </c>
-      <c r="E2" s="28" t="n">
+      <c r="C10" s="38" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D10" s="38" t="inlineStr">
+        <is>
+          <t>Couple</t>
+        </is>
+      </c>
+      <c r="E10" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="38" t="n">
         <v>2</v>
       </c>
-      <c r="F2" s="27" t="n">
+      <c r="H10" s="40" t="inlineStr">
+        <is>
+          <t>R1 w/Rhon,  R5★ w/Alexis,  R9★ w/Alexis</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="38" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="39" t="inlineStr">
+        <is>
+          <t>Richard</t>
+        </is>
+      </c>
+      <c r="C11" s="38" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D11" s="38" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E11" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" s="38" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" s="38" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="27" t="n">
+      <c r="H11" s="40" t="inlineStr">
+        <is>
+          <t>R1 w/Joe,  R3 w/Jay,  R6 w/Arman</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="41" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="42" t="inlineStr">
+        <is>
+          <t>Rhon</t>
+        </is>
+      </c>
+      <c r="C12" s="41" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D12" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E12" s="42" t="n">
+        <v>4</v>
+      </c>
+      <c r="F12" s="41" t="n">
+        <v>4</v>
+      </c>
+      <c r="G12" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="43" t="inlineStr">
+        <is>
+          <t>R1 w/Trevor,  R3 w/Joe,  R5 w/Jay,  R8 w/Jon</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="41" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="42" t="inlineStr">
+        <is>
+          <t>Joe</t>
+        </is>
+      </c>
+      <c r="C13" s="41" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D13" s="41" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E13" s="42" t="n">
+        <v>4</v>
+      </c>
+      <c r="F13" s="41" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" s="41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="43" t="inlineStr">
+        <is>
+          <t>R1 w/Richard,  R3 w/Rhon,  R6 w/Jon,  R8 w/Arman</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="38" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="39" t="inlineStr">
+        <is>
+          <t>Pierre</t>
+        </is>
+      </c>
+      <c r="C14" s="38" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D14" s="38" t="inlineStr">
+        <is>
+          <t>Couple</t>
+        </is>
+      </c>
+      <c r="E14" s="39" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" s="38" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="38" t="n">
         <v>2</v>
       </c>
-      <c r="H2" s="29" t="inlineStr">
-        <is>
-          <t>Trevor (R4-N★),  Trevor (R7-S★)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="27" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="28" t="inlineStr">
-        <is>
-          <t>Carmela</t>
-        </is>
-      </c>
-      <c r="C3" s="27" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D3" s="27" t="inlineStr">
-        <is>
-          <t>Marv</t>
-        </is>
-      </c>
-      <c r="E3" s="28" t="n">
-        <v>3</v>
-      </c>
-      <c r="F3" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="27" t="n">
-        <v>3</v>
-      </c>
-      <c r="H3" s="29" t="inlineStr">
-        <is>
-          <t>Marv (R4-S★),  Marv (R5-S★),  Marv (R9-N★)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="27" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="28" t="inlineStr">
-        <is>
-          <t>Ivy</t>
-        </is>
-      </c>
-      <c r="C4" s="27" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="D4" s="27" t="inlineStr">
-        <is>
-          <t>Pierre</t>
-        </is>
-      </c>
-      <c r="E4" s="28" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" s="27" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="27" t="n">
-        <v>2</v>
-      </c>
-      <c r="H4" s="29" t="inlineStr">
-        <is>
-          <t>Pierre (R7-N★),  Pierre (R9-S★)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="30" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="31" t="inlineStr">
-        <is>
-          <t>Jay</t>
-        </is>
-      </c>
-      <c r="C5" s="30" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D5" s="30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E5" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="F5" s="30" t="n">
-        <v>3</v>
-      </c>
-      <c r="G5" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="32" t="inlineStr">
-        <is>
-          <t>Rhon (R2-N),  Richard (R3-S),  Joe (R6-S)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="30" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="31" t="inlineStr">
-        <is>
-          <t>Marv</t>
-        </is>
-      </c>
-      <c r="C6" s="30" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D6" s="30" t="inlineStr">
-        <is>
-          <t>Carmela</t>
-        </is>
-      </c>
-      <c r="E6" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="F6" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="30" t="n">
-        <v>3</v>
-      </c>
-      <c r="H6" s="32" t="inlineStr">
-        <is>
-          <t>Carmela (R4-S★),  Carmela (R5-S★),  Carmela (R9-N★)</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="33" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="34" t="inlineStr">
-        <is>
-          <t>Arman</t>
-        </is>
-      </c>
-      <c r="C7" s="33" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D7" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E7" s="34" t="n">
-        <v>4</v>
-      </c>
-      <c r="F7" s="33" t="n">
-        <v>4</v>
-      </c>
-      <c r="G7" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="35" t="inlineStr">
-        <is>
-          <t>Rhon (R1-S),  Joe (R2-S),  Pierre (R3-N),  Richard (R5-N)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="30" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="31" t="inlineStr">
-        <is>
-          <t>Jon</t>
-        </is>
-      </c>
-      <c r="C8" s="30" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D8" s="30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E8" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="F8" s="30" t="n">
-        <v>3</v>
-      </c>
-      <c r="G8" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="32" t="inlineStr">
-        <is>
-          <t>Richard (R1-N),  Trevor (R6-N),  Joe (R8-N)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="30" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="31" t="inlineStr">
-        <is>
-          <t>Trevor</t>
-        </is>
-      </c>
-      <c r="C9" s="30" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D9" s="30" t="inlineStr">
-        <is>
-          <t>Alexis</t>
-        </is>
-      </c>
-      <c r="E9" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="F9" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="30" t="n">
-        <v>2</v>
-      </c>
-      <c r="H9" s="32" t="inlineStr">
-        <is>
-          <t>Alexis (R4-N★),  Jon (R6-N),  Alexis (R7-S★)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="33" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="34" t="inlineStr">
-        <is>
-          <t>Richard</t>
-        </is>
-      </c>
-      <c r="C10" s="33" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D10" s="33" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E10" s="34" t="n">
-        <v>4</v>
-      </c>
-      <c r="F10" s="33" t="n">
-        <v>4</v>
-      </c>
-      <c r="G10" s="33" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="35" t="inlineStr">
-        <is>
-          <t>Jon (R1-N),  Jay (R3-S),  Arman (R5-N),  Rhon (R8-S)</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="30" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="31" t="inlineStr">
-        <is>
-          <t>Rhon</t>
-        </is>
-      </c>
-      <c r="C11" s="30" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D11" s="30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E11" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="F11" s="30" t="n">
-        <v>3</v>
-      </c>
-      <c r="G11" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="32" t="inlineStr">
-        <is>
-          <t>Arman (R1-S),  Jay (R2-N),  Richard (R8-S)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="30" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="31" t="inlineStr">
-        <is>
-          <t>Joe</t>
-        </is>
-      </c>
-      <c r="C12" s="30" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D12" s="30" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E12" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="F12" s="30" t="n">
-        <v>3</v>
-      </c>
-      <c r="G12" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" s="32" t="inlineStr">
-        <is>
-          <t>Arman (R2-S),  Jay (R6-S),  Jon (R8-N)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="30" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="31" t="inlineStr">
-        <is>
-          <t>Pierre</t>
-        </is>
-      </c>
-      <c r="C13" s="30" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="D13" s="30" t="inlineStr">
-        <is>
-          <t>Ivy</t>
-        </is>
-      </c>
-      <c r="E13" s="31" t="n">
-        <v>3</v>
-      </c>
-      <c r="F13" s="30" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" s="30" t="n">
-        <v>2</v>
-      </c>
-      <c r="H13" s="32" t="inlineStr">
-        <is>
-          <t>Arman (R3-N),  Ivy (R7-N★),  Ivy (R9-S★)</t>
+      <c r="H14" s="40" t="inlineStr">
+        <is>
+          <t>R2 w/Arman,  R4★ w/Ivy,  R7★ w/Ivy</t>
         </is>
       </c>
     </row>

</xml_diff>